<commit_message>
Fix: initialise Config dictionary, remove blank row in Settings sheet
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WebProgApps\CarbonEmissionsVehicleChecker\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WebProgApps\CarbonEmissionsVehicleChecker_v2\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F111D10-CB1E-46EA-882B-C8AEF8A25E16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2E5B03A-C29C-4FF0-BC9E-3B9486E9EFD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="750" yWindow="220" windowWidth="18030" windowHeight="11060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -615,7 +615,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z998"/>
+  <dimension ref="A1:Z997"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="29.54296875" customWidth="1"/>
@@ -676,62 +676,62 @@
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="29">
+    <row r="4" spans="1:26" ht="29">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" ht="14.25" customHeight="1">
       <c r="A5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" t="s">
-        <v>41</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>21</v>
+        <v>42</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1">
       <c r="A6" t="s">
-        <v>42</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="C6" t="s">
-        <v>44</v>
+        <v>45</v>
+      </c>
+      <c r="B6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" t="s">
-        <v>45</v>
-      </c>
-      <c r="B7" t="s">
-        <v>46</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
       <c r="A8" t="s">
-        <v>48</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C8" t="s">
-        <v>50</v>
+        <v>51</v>
+      </c>
+      <c r="B8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>53</v>
       </c>
     </row>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A9" t="s">
-        <v>51</v>
-      </c>
-      <c r="B9" t="s">
-        <v>52</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
+    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
@@ -1720,12 +1720,11 @@
     <row r="995" ht="14.25" customHeight="1"/>
     <row r="996" ht="14.25" customHeight="1"/>
     <row r="997" ht="14.25" customHeight="1"/>
-    <row r="998" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1" xr:uid="{7D4BE315-4DA0-499B-B209-3F0C17AE4460}"/>
-    <hyperlink ref="B8" r:id="rId2" xr:uid="{4350E108-10A3-4EEF-9AEB-126FD71A9EC2}"/>
+    <hyperlink ref="B5" r:id="rId1" xr:uid="{7D4BE315-4DA0-499B-B209-3F0C17AE4460}"/>
+    <hyperlink ref="B7" r:id="rId2" xr:uid="{4350E108-10A3-4EEF-9AEB-126FD71A9EC2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>

</xml_diff>

<commit_message>
ScrapeData: navigate to Low Emissions search page (skipped dropdown)
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WebProgApps\CarbonEmissionsVehicleChecker_v2\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2E5B03A-C29C-4FF0-BC9E-3B9486E9EFD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3623CFDF-FD3B-4280-889A-0C12151DD87E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="750" yWindow="220" windowWidth="18030" windowHeight="11060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="750" yWindow="220" windowWidth="18030" windowHeight="11060" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -1733,7 +1733,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Z988"/>
+  <dimension ref="A1:Z984"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
@@ -1798,186 +1798,186 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="4" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+    </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>13</v>
+      </c>
+    </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="C10" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
       <c r="A11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" t="s">
-        <v>19</v>
+        <v>32</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
       </c>
       <c r="C11" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
-        <v>31</v>
-      </c>
-      <c r="B12" t="s">
-        <v>40</v>
+        <v>33</v>
+      </c>
+      <c r="B12">
+        <v>2</v>
       </c>
       <c r="C12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="13" spans="1:26" ht="29">
+      <c r="A13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
-        <v>32</v>
+        <v>54</v>
       </c>
       <c r="B14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C14" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="B15">
-        <v>2</v>
+        <v>2000</v>
       </c>
       <c r="C15" t="s">
-        <v>36</v>
+        <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" spans="1:3" ht="29">
+    <row r="16" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A16" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16">
+        <v>100</v>
+      </c>
+      <c r="C16" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="14.25" customHeight="1">
       <c r="A17" t="s">
-        <v>37</v>
-      </c>
-      <c r="B17" t="b">
-        <v>1</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>39</v>
+        <v>60</v>
+      </c>
+      <c r="B17">
+        <v>30000</v>
+      </c>
+      <c r="C17" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1">
       <c r="A18" t="s">
-        <v>54</v>
-      </c>
-      <c r="B18">
-        <v>3</v>
+        <v>62</v>
+      </c>
+      <c r="B18" t="s">
+        <v>63</v>
       </c>
       <c r="C18" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="14.25" customHeight="1">
       <c r="A19" t="s">
-        <v>56</v>
-      </c>
-      <c r="B19">
-        <v>2000</v>
+        <v>65</v>
+      </c>
+      <c r="B19" t="s">
+        <v>66</v>
       </c>
       <c r="C19" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A20" t="s">
-        <v>58</v>
-      </c>
-      <c r="B20">
-        <v>100</v>
-      </c>
-      <c r="C20" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A21" t="s">
-        <v>60</v>
-      </c>
-      <c r="B21">
-        <v>30000</v>
-      </c>
-      <c r="C21" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A22" t="s">
-        <v>62</v>
-      </c>
-      <c r="B22" t="s">
-        <v>63</v>
-      </c>
-      <c r="C22" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A23" t="s">
-        <v>65</v>
-      </c>
-      <c r="B23" t="s">
-        <v>66</v>
-      </c>
-      <c r="C23" t="s">
-        <v>67</v>
-      </c>
-    </row>
+    <row r="20" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="21" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="22" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="23" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="24" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="25" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="26" spans="1:3" ht="14.25" customHeight="1"/>
@@ -2939,10 +2939,6 @@
     <row r="982" ht="14.25" customHeight="1"/>
     <row r="983" ht="14.25" customHeight="1"/>
     <row r="984" ht="14.25" customHeight="1"/>
-    <row r="985" ht="14.25" customHeight="1"/>
-    <row r="986" ht="14.25" customHeight="1"/>
-    <row r="987" ht="14.25" customHeight="1"/>
-    <row r="988" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>